<commit_message>
fixed the routing and added the delivery data
</commit_message>
<xml_diff>
--- a/Distance/geocache.xlsx
+++ b/Distance/geocache.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1164,6 +1164,24 @@
         <v>2.336469</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Hôtel Dieu Hospital</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1 Parvis Notre-Dame - Place Jean-Paul II, 75004 Paris, France</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>48.853888</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2.348293</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>